<commit_message>
docs: exclude workbook changes from pull request
Restore the workbook in the branch to its main version while keeping the updated local workbook uncommitted.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
Copilot-Session: e9201403-8dc7-4208-aa91-c5d525cf083f
</commit_message>
<xml_diff>
--- a/demo/rubric-simulator.xlsx
+++ b/demo/rubric-simulator.xlsx
@@ -1,208 +1,99 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
-  <workbookPr filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="점수표" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="점수표" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
-  <si>
-    <t>급식배틀 루브릭 시뮬레이터</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>노란 셀(학교 이름 · 현재 가중치 · 점수)을 바꾸면 총점과 승자가 다시 계산됩니다</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>평가 영역</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>가중치</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>점수 (1~5)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>환산 점수 (100점 만점)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>기본</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>현재</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>부광고등학교</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>용강초등학교</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>영양·건강성</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>식재료 품질·안전성</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>메뉴 다양성·기호도</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>지속가능성·가격 가치</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>합계</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>승부 결과</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>항목</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>기본 가중치</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>현재 가중치</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>변화</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>승자</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>점수 차</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>계산 방식</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>• 앱 공식 (rubric.py): 영역 환산 점수 = 획득 점수 ÷ 5 × 가중치, 총점 = 네 영역의 합</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>• 현재 가중치 합계가 100이 아니어도 100점 만점으로 정규화해 비교합니다</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>• 브라우저의 완료된 분석 결과에서 옮긴 점수입니다. 분석 대상 날짜와 상세 평가 근거는 제공된 화면에 없어 포함하지 않았습니다.</t>
-    <phoneticPr fontId="1"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="20"/>
-      <color rgb="00FFFFFF"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <i/>
+      <name val="Malgun Gothic"/>
+      <i val="1"/>
+      <color rgb="006B6B6B"/>
       <sz val="10"/>
-      <color rgb="006B6B6B"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
-      <color rgb="00FFFFFF"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00222222"/>
       <sz val="11"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
+      <name val="Malgun Gothic"/>
+      <color rgb="00222222"/>
       <sz val="11"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
+      <name val="Malgun Gothic"/>
+      <color rgb="006B6B6B"/>
       <sz val="11"/>
-      <color rgb="006B6B6B"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00222222"/>
       <sz val="12"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="13"/>
-      <color rgb="00FFFFFF"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
+      <name val="Malgun Gothic"/>
+      <color rgb="00222222"/>
       <sz val="12"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00222222"/>
       <sz val="14"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
-      <b/>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
+      <color rgb="00222222"/>
       <sz val="10"/>
-      <color rgb="00222222"/>
-      <name val="Malgun Gothic"/>
     </font>
     <font>
+      <name val="Malgun Gothic"/>
+      <color rgb="006B6B6B"/>
       <sz val="10"/>
-      <color rgb="006B6B6B"/>
-      <name val="Malgun Gothic"/>
     </font>
   </fonts>
   <fills count="7">
@@ -259,81 +150,80 @@
       <bottom style="thin">
         <color rgb="00B7C4B7"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color rgb="00E8590C"/>
       </font>
       <fill>
@@ -344,19 +234,19 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color rgb="00E8590C"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color rgb="0037734C"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color rgb="00FFFFFF"/>
       </font>
       <fill>
@@ -366,12 +256,75 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -576,10 +529,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -610,10 +563,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -650,20 +603,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
                 <a:satMod val="300000"/>
-                <a:tint val="50000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
                 <a:satMod val="300000"/>
-                <a:tint val="37000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
-                <a:tint val="15000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -673,20 +626,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
-                <a:shade val="51000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
                 <a:satMod val="130000"/>
-                <a:shade val="93000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
                 <a:satMod val="135000"/>
-                <a:shade val="94000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -697,8 +650,8 @@
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
               <a:satMod val="105000"/>
-              <a:shade val="95000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
@@ -764,40 +717,46 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
                 <a:satMod val="350000"/>
-                <a:tint val="40000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
                 <a:satMod val="350000"/>
-                <a:shade val="99000"/>
-                <a:tint val="45000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
                 <a:satMod val="255000"/>
-                <a:shade val="20000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
-                <a:tint val="80000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
-                <a:shade val="30000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -808,312 +767,371 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="3" width="10" customWidth="1"/>
-    <col min="4" max="5" width="13" customWidth="1"/>
-    <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="3" customWidth="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="40" customHeight="1">
-      <c r="A1" t="s" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="22" customHeight="1">
-      <c r="A2" t="s" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="24" customHeight="1">
-      <c r="A3" t="s" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="3">
-        <v>3</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" t="s" s="3">
-        <v>4</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" t="s" s="3">
-        <v>5</v>
-      </c>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" ht="24" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" t="s" s="5">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s" s="5">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s" s="6">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s" s="6">
-        <v>9</v>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>급식배틀 루브릭 시뮬레이터</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>노란 셀(학교 이름 · 현재 가중치 · 점수)을 바꾸면 총점과 승자가 다시 계산됩니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>평가 영역</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>가중치</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>점수 (1~5)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>환산 점수 (100점 만점)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>기본</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>현재</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>학교 A</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>학교 B</t>
+        </is>
       </c>
       <c r="F4" s="5" t="str">
         <f>D4</f>
-        <v>부광고등학교</v>
+        <v>학교 A</v>
       </c>
       <c r="G4" s="5" t="str">
         <f>E4</f>
-        <v>용강초등학교</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="24" customHeight="1">
-      <c r="A5" t="s" s="7">
-        <v>10</v>
-      </c>
-      <c r="B5" s="8">
+        <v>학교 B</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>영양·건강성</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="6">
-        <v>3</v>
-      </c>
-      <c r="E5" s="6">
+      <c r="D5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="9">
         <f>ROUND(D5/5*C5/C9*100,2)</f>
-        <v>21.0</v>
+        <v>35</v>
       </c>
       <c r="G5" s="9">
         <f>ROUND(E5/5*C5/C9*100,2)</f>
-        <v>21.0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="24" customHeight="1">
-      <c r="A6" t="s" s="7">
-        <v>11</v>
-      </c>
-      <c r="B6" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>식재료 품질·안전성</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="E6" s="6">
-        <v>3</v>
       </c>
       <c r="F6" s="9">
         <f>ROUND(D6/5*C6/C9*100,2)</f>
-        <v>20.0</v>
+        <v>15</v>
       </c>
       <c r="G6" s="9">
         <f>ROUND(E6/5*C6/C9*100,2)</f>
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" t="s" s="7">
-        <v>12</v>
-      </c>
-      <c r="B7" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>메뉴 다양성·기호도</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="D7" s="6">
-        <v>4</v>
-      </c>
-      <c r="E7" s="6">
+      <c r="D7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="F7" s="9">
         <f>ROUND(D7/5*C7/C9*100,2)</f>
-        <v>20.0</v>
+        <v>15</v>
       </c>
       <c r="G7" s="9">
         <f>ROUND(E7/5*C7/C9*100,2)</f>
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="24" customHeight="1">
-      <c r="A8" t="s" s="7">
-        <v>13</v>
-      </c>
-      <c r="B8" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>지속가능성·가격 가치</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="6">
-        <v>3</v>
-      </c>
-      <c r="E8" s="6">
-        <v>4</v>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="F8" s="9">
         <f>ROUND(D8/5*C8/C9*100,2)</f>
-        <v>9.0</v>
+        <v>6</v>
       </c>
       <c r="G8" s="9">
         <f>ROUND(E8/5*C8/C9*100,2)</f>
-        <v>12.0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="26" customHeight="1">
-      <c r="A9" t="s" s="10">
-        <v>14</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
       </c>
       <c r="B9" s="11">
         <f>SUM(B5:B8)</f>
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="C9" s="11">
         <f>SUM(C5:C8)</f>
-        <v>100.0</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
+        <v>100</v>
+      </c>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
       <c r="F9" s="12">
         <f>ROUND(SUM(F5:F8),2)</f>
-        <v>70.0</v>
+        <v>71</v>
       </c>
       <c r="G9" s="12">
         <f>ROUND(SUM(G5:G8),2)</f>
-        <v>68.0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="28" customHeight="1">
-      <c r="A11" t="s" s="13">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="24" customHeight="1">
-      <c r="A12" t="s" s="5">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" t="s" s="5">
-        <v>18</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" t="s" s="5">
-        <v>19</v>
-      </c>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" ht="26" customHeight="1">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>승부 결과</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>기본 가중치</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>현재 가중치</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>변화</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
       <c r="A13" s="14" t="str">
         <f>CONCATENATE(D4," 총점")</f>
-        <v>부광고등학교 총점</v>
+        <v>학교 A 총점</v>
       </c>
       <c r="B13" s="15">
         <f>ROUND(SUMPRODUCT(D5:D8,B5:B8)/5/B9*100,2)</f>
-        <v>70.0</v>
-      </c>
-      <c r="C13" s="16"/>
+        <v>71</v>
+      </c>
+      <c r="C13" s="16" t="n"/>
       <c r="D13" s="15">
         <f>F9</f>
-        <v>70.0</v>
-      </c>
-      <c r="E13" s="16"/>
+        <v>71</v>
+      </c>
+      <c r="E13" s="16" t="n"/>
       <c r="F13" s="17">
         <f>ROUND(D13-B13,2)</f>
-        <v>0.0</v>
-      </c>
-      <c r="G13" s="16"/>
-    </row>
-    <row r="14" spans="1:7" ht="26" customHeight="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="16" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
       <c r="A14" s="14" t="str">
         <f>CONCATENATE(E4," 총점")</f>
-        <v>용강초등학교 총점</v>
+        <v>학교 B 총점</v>
       </c>
       <c r="B14" s="15">
         <f>ROUND(SUMPRODUCT(E5:E8,B5:B8)/5/B9*100,2)</f>
-        <v>68.0</v>
-      </c>
-      <c r="C14" s="16"/>
+        <v>76</v>
+      </c>
+      <c r="C14" s="16" t="n"/>
       <c r="D14" s="15">
         <f>G9</f>
-        <v>68.0</v>
-      </c>
-      <c r="E14" s="16"/>
+        <v>76</v>
+      </c>
+      <c r="E14" s="16" t="n"/>
       <c r="F14" s="17">
         <f>ROUND(D14-B14,2)</f>
-        <v>0.0</v>
-      </c>
-      <c r="G14" s="16"/>
-    </row>
-    <row r="15" spans="1:7" ht="32" customHeight="1">
-      <c r="A15" t="s" s="14">
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="G14" s="16" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>승자</t>
+        </is>
       </c>
       <c r="B15" s="18" t="str">
         <f>IF(B13&gt;B14,D4,IF(B14&gt;B13,E4,"동점"))</f>
-        <v>부광고등학교</v>
-      </c>
-      <c r="C15" s="16"/>
+        <v>학교 B</v>
+      </c>
+      <c r="C15" s="16" t="n"/>
       <c r="D15" s="19" t="str">
         <f>IF(D13&gt;D14,D4,IF(D14&gt;D13,E4,"동점"))</f>
-        <v>부광고등학교</v>
-      </c>
-      <c r="E15" s="16"/>
+        <v>학교 B</v>
+      </c>
+      <c r="E15" s="16" t="n"/>
       <c r="F15" s="18" t="str">
         <f>IF(B15=D15,"그대로","뒤집힘!")</f>
         <v>그대로</v>
       </c>
-      <c r="G15" s="16"/>
-    </row>
-    <row r="16" spans="1:7" ht="26" customHeight="1">
-      <c r="A16" t="s" s="14">
-        <v>21</v>
+      <c r="G15" s="16" t="n"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>점수 차</t>
+        </is>
       </c>
       <c r="B16" s="15">
         <f>ROUND(ABS(B13-B14),2)</f>
-        <v>2.0</v>
-      </c>
-      <c r="C16" s="16"/>
+        <v>5</v>
+      </c>
+      <c r="C16" s="16" t="n"/>
       <c r="D16" s="15">
         <f>ROUND(ABS(D13-D14),2)</f>
-        <v>2.0</v>
-      </c>
-      <c r="E16" s="16"/>
+        <v>5</v>
+      </c>
+      <c r="E16" s="16" t="n"/>
       <c r="F16" s="17">
         <f>ROUND(D16-B16,2)</f>
-        <v>0.0</v>
-      </c>
-      <c r="G16" s="16"/>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s" s="20">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s" s="21">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" t="s" s="21">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" t="s" s="21">
-        <v>25</v>
+        <v>0</v>
+      </c>
+      <c r="G16" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>계산 방식</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>• 앱 공식 (rubric.py): 영역 환산 점수 = 획득 점수 ÷ 5 × 가중치, 총점 = 네 영역의 합</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>• 현재 가중치 합계가 100이 아니어도 100점 만점으로 정규화해 비교합니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>• 예시 점수는 데모용입니다. 무대에서 실제 분석 결과(영역별 1~5점)로 덮어쓰세요</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1141,42 +1159,42 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="F14:G14"/>
   </mergeCells>
-  <phoneticPr fontId="1"/>
   <conditionalFormatting sqref="C5:C8">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>C5&lt;&gt;B5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" priority="2" dxfId="1">
       <formula>C9&lt;&gt;100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F9">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" priority="3" dxfId="2">
       <formula>F5&gt;G5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G9">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" priority="4" dxfId="2">
       <formula>G5&gt;F5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F15">
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" priority="5" dxfId="3">
       <formula>F15="뒤집힘!"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="0" showInputMessage="1" operator="between" showErrorMessage="1" errorTitle="&amp;#51216;&amp;#49688; &amp;#48276;&amp;#50948;" error="&amp;#51216;&amp;#49688;&amp;#45716; 1~5 &amp;#49324;&amp;#51060; &amp;#51221;&amp;#49688;&amp;#47196; &amp;#51077;&amp;#47141;&amp;#54616;&amp;#49464;&amp;#50836;" promptTitle="&amp;#51216;&amp;#49688;" prompt="1~5 &amp;#49324;&amp;#51060; &amp;#51221;&amp;#49688;" sqref="D5:E8">
+    <dataValidation sqref="D5:E8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="점수 범위" error="점수는 1~5 사이 정수로 입력하세요" promptTitle="점수" prompt="1~5 사이 정수" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="0" showInputMessage="1" operator="between" showErrorMessage="1" errorTitle="&amp;#44032;&amp;#51473;&amp;#52824; &amp;#48276;&amp;#50948;" error="&amp;#44032;&amp;#51473;&amp;#52824;&amp;#45716; 0~100 &amp;#49324;&amp;#51060; &amp;#51221;&amp;#49688;&amp;#47196; &amp;#51077;&amp;#47141;&amp;#54616;&amp;#49464;&amp;#50836;" promptTitle="&amp;#44032;&amp;#51473;&amp;#52824;" prompt="0~100 &amp;#49324;&amp;#51060; &amp;#51221;&amp;#49688;" sqref="C5:C8">
+    <dataValidation sqref="C5:C8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="가중치 범위" error="가중치는 0~100 사이 정수로 입력하세요" promptTitle="가중치" prompt="0~100 사이 정수" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>